<commit_message>
Margin top-30: salt cost 4500 RUB/t
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/MARGIN_TOP30_1210.xlsx
+++ b/MARGIN_TOP30_1210.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>УСН 15%: прибыль = цена − себестоимость − 0,8% прочих − стоимость денег 20% годовых × 60 дн., минус налог 15% с прибыли. Себестоимость соли 2 500 ₽/т с доставкой (без последней мили).</t>
+          <t>УСН 15%: прибыль = цена − себестоимость − 0,8% прочих − стоимость денег 20% годовых × 60 дн., минус налог 15% с прибыли. Себестоимость соли 4 500 ₽/т с доставкой.</t>
         </is>
       </c>
     </row>
@@ -667,27 +667,27 @@
         <v>13869240</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2370000</v>
+        <v>4266000</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>948 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>948 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.8291182501708817</v>
+        <v>0.6924128503075871</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>9613813</v>
+        <v>7949229</v>
       </c>
       <c r="L4" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>7859632</v>
+        <v>6195047</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>0.8220768347172515</v>
+        <v>0.6797383024910526</v>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
     </row>
@@ -724,27 +724,27 @@
         <v>6724000</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1000000</v>
+        <v>1800000</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>400 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>400 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.851279000594884</v>
+        <v>0.7323022010707912</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>4791732</v>
+        <v>4089375</v>
       </c>
       <c r="L5" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>3941280</v>
+        <v>3238924</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.8451507490727774</v>
+        <v>0.7212713483309994</v>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
     </row>
@@ -781,27 +781,27 @@
         <v>1593800</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>325000</v>
+        <v>585000</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>130 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>130 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.7960848287112561</v>
+        <v>0.632952691680261</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>1058560</v>
+        <v>830294</v>
       </c>
       <c r="L6" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>856976</v>
+        <v>628710</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>0.7876822260940773</v>
+        <v>0.6178280069693394</v>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
     </row>
@@ -887,27 +887,27 @@
         <v>4400000</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1000000</v>
+        <v>1800000</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>400 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>400 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2832135</v>
+        <v>2129779</v>
       </c>
       <c r="L8" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2275623</v>
+        <v>1573267</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>0.7633621901739445</v>
+        <v>0.5740519423131</v>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
     </row>
@@ -944,27 +944,27 @@
         <v>1368000</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>375000</v>
+        <v>675000</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>150 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>150 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.7258771929824561</v>
+        <v>0.506578947368421</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>824268</v>
+        <v>560885</v>
       </c>
       <c r="L9" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>651244</v>
+        <v>387860</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.7145815890255909</v>
+        <v>0.4862468602460637</v>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
     </row>
@@ -1001,27 +1001,27 @@
         <v>3450000</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>862500</v>
+        <v>1552500</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>345 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>345 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2151812</v>
+        <v>1546030</v>
       </c>
       <c r="L10" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1715456</v>
+        <v>1109674</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>0.7396984091913389</v>
+        <v>0.53145713654441</v>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
     </row>
@@ -1058,27 +1058,27 @@
         <v>106470</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>21250</v>
+        <v>34250</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>6,5 т × 2 500 ₽ + фасовка в мешки 5 000 ₽ [оценка]</t>
+          <t>6,5 т × 4 500 ₽ + фасовка в мешки 5 000 ₽ [оценка]</t>
         </is>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.8004132619517235</v>
+        <v>0.6783131398516014</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>71119</v>
+        <v>59706</v>
       </c>
       <c r="L11" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>57653</v>
+        <v>46240</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>0.7921890183268884</v>
+        <v>0.6650575942445143</v>
       </c>
       <c r="O11" s="3" t="inlineStr"/>
     </row>
@@ -1115,27 +1115,27 @@
         <v>121000000</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>27500000</v>
+        <v>49500000</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>11000 т × 2 500 ₽ (Казахстан, с доставкой)</t>
+          <t>11000 т × 4 500 ₽ (с доставкой)</t>
         </is>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>77883707</v>
+        <v>58568912</v>
       </c>
       <c r="L12" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>62579627</v>
+        <v>43264832</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.7633621901739445</v>
+        <v>0.5740519423131001</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -2384,16 +2384,16 @@
         <v>152511510</v>
       </c>
       <c r="H35" s="19" t="n">
-        <v>33453750</v>
+        <v>60212750</v>
       </c>
       <c r="I35" s="18" t="inlineStr"/>
       <c r="J35" s="20" t="n"/>
       <c r="K35" s="19" t="n">
-        <v>99227146</v>
+        <v>75734210</v>
       </c>
       <c r="L35" s="20" t="inlineStr"/>
       <c r="M35" s="19" t="n">
-        <v>79937491</v>
+        <v>56444554</v>
       </c>
       <c r="N35" s="20" t="inlineStr"/>
       <c r="O35" s="18" t="inlineStr"/>
@@ -2558,16 +2558,16 @@
         <v>62392848</v>
       </c>
       <c r="H41" s="19" t="n">
-        <v>22154582</v>
+        <v>26913582</v>
       </c>
       <c r="I41" s="18" t="inlineStr"/>
       <c r="J41" s="20" t="n"/>
       <c r="K41" s="19" t="n">
-        <v>33159142</v>
+        <v>28981001</v>
       </c>
       <c r="L41" s="20" t="inlineStr"/>
       <c r="M41" s="19" t="n">
-        <v>24626247</v>
+        <v>20448105</v>
       </c>
       <c r="N41" s="20" t="inlineStr"/>
       <c r="O41" s="18" t="inlineStr"/>
@@ -2587,16 +2587,16 @@
         <v>183392848</v>
       </c>
       <c r="H42" s="19" t="n">
-        <v>49654582</v>
+        <v>76413582</v>
       </c>
       <c r="I42" s="18" t="inlineStr"/>
       <c r="J42" s="20" t="n"/>
       <c r="K42" s="19" t="n">
-        <v>111042849</v>
+        <v>87549913</v>
       </c>
       <c r="L42" s="20" t="inlineStr"/>
       <c r="M42" s="19" t="n">
-        <v>87205874</v>
+        <v>63712937</v>
       </c>
       <c r="N42" s="20" t="inlineStr"/>
       <c r="O42" s="18" t="inlineStr"/>

</xml_diff>

<commit_message>
Top-30 tables: ruble number format with thousand separators, autofilter on data rows, totals on separate sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/MARGIN_TOP30_1210.xlsx
+++ b/MARGIN_TOP30_1210.xlsx
@@ -8,8 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Маржа топ-30" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Маржа топ-30'!$A$3:$O$33</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="# ##0"/>
+    <numFmt numFmtId="164" formatCode="#,##0&quot; ₽&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -149,15 +152,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,23 +520,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="36" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -2352,254 +2349,236 @@
       </c>
       <c r="O33" s="12" t="inlineStr"/>
     </row>
-    <row r="34">
-      <c r="A34" s="15" t="n"/>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
-      <c r="I34" s="15" t="n"/>
-      <c r="J34" s="17" t="n"/>
-      <c r="K34" s="16" t="n"/>
-      <c r="L34" s="17" t="n"/>
-      <c r="M34" s="16" t="n"/>
-      <c r="N34" s="17" t="n"/>
-      <c r="O34" s="15" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="18" t="inlineStr"/>
-      <c r="B35" s="18" t="inlineStr"/>
-      <c r="C35" s="18" t="inlineStr">
-        <is>
-          <t>Итого: Соль</t>
-        </is>
-      </c>
-      <c r="D35" s="18" t="inlineStr"/>
-      <c r="E35" s="18" t="inlineStr"/>
-      <c r="F35" s="18" t="inlineStr"/>
-      <c r="G35" s="19" t="n">
+  </sheetData>
+  <autoFilter ref="A3:O33"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Лотов</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>НМЦК, ₽</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Себестоимость, ₽</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Чистая прибыль при НМЦК, ₽</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Чистая прибыль при ожид. снижении, ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Соль</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="18" t="n">
         <v>152511510</v>
       </c>
-      <c r="H35" s="19" t="n">
+      <c r="D2" s="18" t="n">
         <v>60212750</v>
       </c>
-      <c r="I35" s="18" t="inlineStr"/>
-      <c r="J35" s="20" t="n"/>
-      <c r="K35" s="19" t="n">
+      <c r="E2" s="18" t="n">
         <v>75734210</v>
       </c>
-      <c r="L35" s="20" t="inlineStr"/>
-      <c r="M35" s="19" t="n">
+      <c r="F2" s="18" t="n">
         <v>56444554</v>
       </c>
-      <c r="N35" s="20" t="inlineStr"/>
-      <c r="O35" s="18" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr"/>
-      <c r="B36" s="18" t="inlineStr"/>
-      <c r="C36" s="18" t="inlineStr">
-        <is>
-          <t>Итого: ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="D36" s="18" t="inlineStr"/>
-      <c r="E36" s="18" t="inlineStr"/>
-      <c r="F36" s="18" t="inlineStr"/>
-      <c r="G36" s="19" t="n">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="18" t="n">
         <v>4479513</v>
       </c>
-      <c r="H36" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>2117274</v>
       </c>
-      <c r="I36" s="18" t="inlineStr"/>
-      <c r="J36" s="20" t="n"/>
-      <c r="K36" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>1918275</v>
       </c>
-      <c r="L36" s="20" t="inlineStr"/>
-      <c r="M36" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1351706</v>
       </c>
-      <c r="N36" s="20" t="inlineStr"/>
-      <c r="O36" s="18" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="18" t="inlineStr"/>
-      <c r="B37" s="18" t="inlineStr"/>
-      <c r="C37" s="18" t="inlineStr">
-        <is>
-          <t>Итого: Форменная одежда</t>
-        </is>
-      </c>
-      <c r="D37" s="18" t="inlineStr"/>
-      <c r="E37" s="18" t="inlineStr"/>
-      <c r="F37" s="18" t="inlineStr"/>
-      <c r="G37" s="19" t="n">
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Форменная одежда</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="18" t="n">
         <v>11223423</v>
       </c>
-      <c r="H37" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>6001300</v>
       </c>
-      <c r="I37" s="18" t="inlineStr"/>
-      <c r="J37" s="20" t="n"/>
-      <c r="K37" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>4194777</v>
       </c>
-      <c r="L37" s="20" t="inlineStr"/>
-      <c r="M37" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>2775239</v>
       </c>
-      <c r="N37" s="20" t="inlineStr"/>
-      <c r="O37" s="18" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="18" t="inlineStr"/>
-      <c r="B38" s="18" t="inlineStr"/>
-      <c r="C38" s="18" t="inlineStr">
-        <is>
-          <t>Итого: Медрасходники</t>
-        </is>
-      </c>
-      <c r="D38" s="18" t="inlineStr"/>
-      <c r="E38" s="18" t="inlineStr"/>
-      <c r="F38" s="18" t="inlineStr"/>
-      <c r="G38" s="19" t="n">
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="18" t="n">
         <v>9366830</v>
       </c>
-      <c r="H38" s="19" t="n">
+      <c r="D5" s="18" t="n">
         <v>4205030</v>
       </c>
-      <c r="I38" s="18" t="inlineStr"/>
-      <c r="J38" s="20" t="n"/>
-      <c r="K38" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>4206327</v>
       </c>
-      <c r="L38" s="20" t="inlineStr"/>
-      <c r="M38" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>2231796</v>
       </c>
-      <c r="N38" s="20" t="inlineStr"/>
-      <c r="O38" s="18" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="18" t="inlineStr"/>
-      <c r="B39" s="18" t="inlineStr"/>
-      <c r="C39" s="18" t="inlineStr">
-        <is>
-          <t>Итого: Сантехника / арматура</t>
-        </is>
-      </c>
-      <c r="D39" s="18" t="inlineStr"/>
-      <c r="E39" s="18" t="inlineStr"/>
-      <c r="F39" s="18" t="inlineStr"/>
-      <c r="G39" s="19" t="n">
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Сантехника / арматура</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="18" t="n">
         <v>1883587</v>
       </c>
-      <c r="H39" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>1273942</v>
       </c>
-      <c r="I39" s="18" t="inlineStr"/>
-      <c r="J39" s="20" t="n"/>
-      <c r="K39" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>469789</v>
       </c>
-      <c r="L39" s="20" t="inlineStr"/>
-      <c r="M39" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>247436</v>
       </c>
-      <c r="N39" s="20" t="inlineStr"/>
-      <c r="O39" s="18" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="18" t="inlineStr"/>
-      <c r="B40" s="18" t="inlineStr"/>
-      <c r="C40" s="18" t="inlineStr">
-        <is>
-          <t>Итого: СС</t>
-        </is>
-      </c>
-      <c r="D40" s="18" t="inlineStr"/>
-      <c r="E40" s="18" t="inlineStr"/>
-      <c r="F40" s="18" t="inlineStr"/>
-      <c r="G40" s="19" t="n">
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>СС</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="18" t="n">
         <v>3927985</v>
       </c>
-      <c r="H40" s="19" t="n">
+      <c r="D7" s="18" t="n">
         <v>2603286</v>
       </c>
-      <c r="I40" s="18" t="inlineStr"/>
-      <c r="J40" s="20" t="n"/>
-      <c r="K40" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>1026535</v>
       </c>
-      <c r="L40" s="20" t="inlineStr"/>
-      <c r="M40" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>662206</v>
       </c>
-      <c r="N40" s="20" t="inlineStr"/>
-      <c r="O40" s="18" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="18" t="inlineStr"/>
-      <c r="B41" s="18" t="inlineStr"/>
-      <c r="C41" s="18" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>ИТОГО без Самары</t>
         </is>
       </c>
-      <c r="D41" s="18" t="inlineStr"/>
-      <c r="E41" s="18" t="inlineStr"/>
-      <c r="F41" s="18" t="inlineStr"/>
-      <c r="G41" s="19" t="n">
+      <c r="B8" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="20" t="n">
         <v>62392848</v>
       </c>
-      <c r="H41" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>26913582</v>
       </c>
-      <c r="I41" s="18" t="inlineStr"/>
-      <c r="J41" s="20" t="n"/>
-      <c r="K41" s="19" t="n">
+      <c r="E8" s="20" t="n">
         <v>28981001</v>
       </c>
-      <c r="L41" s="20" t="inlineStr"/>
-      <c r="M41" s="19" t="n">
+      <c r="F8" s="20" t="n">
         <v>20448105</v>
       </c>
-      <c r="N41" s="20" t="inlineStr"/>
-      <c r="O41" s="18" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="18" t="inlineStr"/>
-      <c r="B42" s="18" t="inlineStr"/>
-      <c r="C42" s="18" t="inlineStr">
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>ИТОГО с Самарой</t>
         </is>
       </c>
-      <c r="D42" s="18" t="inlineStr"/>
-      <c r="E42" s="18" t="inlineStr"/>
-      <c r="F42" s="18" t="inlineStr"/>
-      <c r="G42" s="19" t="n">
+      <c r="B9" s="19" t="n">
+        <v>29</v>
+      </c>
+      <c r="C9" s="20" t="n">
         <v>183392848</v>
       </c>
-      <c r="H42" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <v>76413582</v>
       </c>
-      <c r="I42" s="18" t="inlineStr"/>
-      <c r="J42" s="20" t="n"/>
-      <c r="K42" s="19" t="n">
+      <c r="E9" s="20" t="n">
         <v>87549913</v>
       </c>
-      <c r="L42" s="20" t="inlineStr"/>
-      <c r="M42" s="19" t="n">
+      <c r="F9" s="20" t="n">
         <v>63712937</v>
       </c>
-      <c r="N42" s="20" t="inlineStr"/>
-      <c r="O42" s="18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>